<commit_message>
30-year PRISM climate data and analysis scripts
</commit_message>
<xml_diff>
--- a/Field_sites_data/Idaho_sites.xlsx
+++ b/Field_sites_data/Idaho_sites.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tshianeondou\Documents\ASW_Lab\Data_Analysis\Field_sites_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tshianeondou\Documents\ASW_Lab\Data_Analysis\Chapter_2\Field_sites_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C49FD97-B434-41DD-90FB-664EF19AAC22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92512153-CE79-4731-80A6-7234B497290D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D41CE469-17B5-4037-A39F-CB294119A5AA}"/>
   </bookViews>
@@ -1092,7 +1092,7 @@
       <c r="AC12" s="24"/>
       <c r="AD12" s="24"/>
     </row>
-    <row r="13" spans="1:30" ht="47" thickBot="1">
+    <row r="13" spans="1:30" ht="31.5" thickBot="1">
       <c r="A13" s="29">
         <v>-116.99</v>
       </c>

</xml_diff>